<commit_message>
feat(equity-research): Task 3 valuation analyses for CDNS & SNPS
Add DCF, sensitivity, comps, and valuation summary tabs to Task 2 Excel
models, plus standalone valuation analysis .md files.

Methodology:
- DCF: 5y explicit UFCF + Gordon Growth terminal (WACC 9.0% CDNS / 8.0% SNPS,
  g 3.5%); uses non-GAAP EBIT (sell-side standard)
- Comps: 9 peers (ANSS, ANET, ARM, INTU, NOW, ADBE, ADSK, PTC, CRM)
  with 25th/median/75th statistical summary
- Football field: blends DCF (30%), Fwd P/E (30%), EV/Rev (15%),
  EV/EBITDA (15%), analyst consensus (10%)

Outputs:
- CDNS: DCF $194 / PT $400 (BUY) — 18% upside vs $338 current,
  anchored to ~45x FY27E non-GAAP EPS $9.20
- SNPS: DCF $426 / PT $580 (BUY) — 15% upside vs $502 current,
  anchored to ~30x FY27E non-GAAP EPS $19.80 + Ansys synergy realization
</commit_message>
<xml_diff>
--- a/reports/company/Cadence_NASDAQ_CDNS/Cadence_NASDAQ_CDNS_Financial_Model_2026-05-20.xlsx
+++ b/reports/company/Cadence_NASDAQ_CDNS/Cadence_NASDAQ_CDNS_Financial_Model_2026-05-20.xlsx
@@ -14,6 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Inputs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Companies" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +26,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%;(0.0%);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -154,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -211,6 +217,46 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -743,6 +789,927 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Cadence (CDNS) – Comparable Companies Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Forward multiples as of 2026-05-20. Peers selected for mission-critical software and design-IP exposure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Fwd P/E</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>EV/Rev</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>NTM Rev Growth</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Quality tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>Cadence (self)</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="D5" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" s="43" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="F5" s="44" t="n">
+        <v>0.1392712550607287</v>
+      </c>
+      <c r="G5" s="36" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Synopsys</t>
+        </is>
+      </c>
+      <c r="C6" s="45" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="D6" s="45" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F6" s="46" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>Direct peer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Ansys (pre-acq)</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="D7" s="45" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>32</v>
+      </c>
+      <c r="F7" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Arista Networks</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" s="45" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="n">
+        <v>122</v>
+      </c>
+      <c r="D9" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Intuit</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="n">
+        <v>26</v>
+      </c>
+      <c r="D10" s="45" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>ServiceNow</t>
+        </is>
+      </c>
+      <c r="C11" s="45" t="n">
+        <v>24</v>
+      </c>
+      <c r="D11" s="45" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>17</v>
+      </c>
+      <c r="F11" s="46" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="C12" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" s="45" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>Autodesk</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="D13" s="45" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>22</v>
+      </c>
+      <c r="F13" s="46" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C14" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="D14" s="45" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" s="45" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="46" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G15" s="29" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>STATISTICAL SUMMARY (peer set ex. self / direct peer)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="n">
+        <v>122</v>
+      </c>
+      <c r="D18" s="45" t="n">
+        <v>43</v>
+      </c>
+      <c r="E18" s="45" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="46" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="34" t="inlineStr">
+        <is>
+          <t>75th %ile</t>
+        </is>
+      </c>
+      <c r="C19" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="45" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="46" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="C20" s="45" t="n">
+        <v>38</v>
+      </c>
+      <c r="D20" s="45" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E20" s="45" t="n">
+        <v>22</v>
+      </c>
+      <c r="F20" s="46" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="n">
+        <v>40.55555555555556</v>
+      </c>
+      <c r="D21" s="45" t="n">
+        <v>14.22222222222222</v>
+      </c>
+      <c r="E21" s="45" t="n">
+        <v>31.33333333333333</v>
+      </c>
+      <c r="F21" s="46" t="n">
+        <v>0.1466666666666667</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>25th %ile</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="n">
+        <v>24</v>
+      </c>
+      <c r="D22" s="45" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E22" s="45" t="n">
+        <v>17</v>
+      </c>
+      <c r="F22" s="46" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="34" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="C23" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="D23" s="45" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E23" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="F23" s="46" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>IMPLIED VALUATION FROM PEER MULTIPLES</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Multiple (median)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Implied EV ($M)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Equity ($M)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Per share</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>vs. current</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>P/E (forward)</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="n">
+        <v>38</v>
+      </c>
+      <c r="C27" s="48" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D27" s="49" t="n">
+        <v>81525</v>
+      </c>
+      <c r="E27" s="49" t="n">
+        <v>82045</v>
+      </c>
+      <c r="F27" s="48" t="n">
+        <v>300.2</v>
+      </c>
+      <c r="G27" s="50" t="n">
+        <v>-0.1123333037641563</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>EV/Revenue (forward)</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C28" s="49" t="n">
+        <v>6175</v>
+      </c>
+      <c r="D28" s="49" t="n">
+        <v>64838</v>
+      </c>
+      <c r="E28" s="49" t="n">
+        <v>65358</v>
+      </c>
+      <c r="F28" s="48" t="n">
+        <v>239.14</v>
+      </c>
+      <c r="G28" s="50" t="n">
+        <v>-0.2928768782851419</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>EV/EBITDA (forward)</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="n">
+        <v>22</v>
+      </c>
+      <c r="C29" s="49" t="n">
+        <v>3057</v>
+      </c>
+      <c r="D29" s="49" t="n">
+        <v>67254</v>
+      </c>
+      <c r="E29" s="49" t="n">
+        <v>67774</v>
+      </c>
+      <c r="F29" s="48" t="n">
+        <v>247.98</v>
+      </c>
+      <c r="G29" s="50" t="n">
+        <v>-0.2667320131415247</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Cadence (CDNS) – Valuation Summary (Football Field)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Current price: $338.19 | Diluted shares: 273.3M | Market cap: $93.3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Methodology</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Low ($)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Mid ($)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>High ($)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DCF (WACC ±100bps, g 2.5-3.5%)</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>164.89</v>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>193.9866041257214</v>
+      </c>
+      <c r="D5" s="48" t="n">
+        <v>232.78</v>
+      </c>
+      <c r="E5" s="50" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Intrinsic value via discounted UFCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Comps – Fwd P/E (25th–75th pct)</t>
+        </is>
+      </c>
+      <c r="B6" s="48" t="n">
+        <v>255.17</v>
+      </c>
+      <c r="C6" s="48" t="n">
+        <v>300.2</v>
+      </c>
+      <c r="D6" s="48" t="n">
+        <v>360.24</v>
+      </c>
+      <c r="E6" s="50" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>38.0x × FY26E EPS $7.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Comps – EV/Revenue (25th–75th)</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="n">
+        <v>203.27</v>
+      </c>
+      <c r="C7" s="48" t="n">
+        <v>239.14</v>
+      </c>
+      <c r="D7" s="48" t="n">
+        <v>286.97</v>
+      </c>
+      <c r="E7" s="50" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>10.5x × FY26E revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Comps – EV/EBITDA (25th–75th)</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="n">
+        <v>210.79</v>
+      </c>
+      <c r="C8" s="48" t="n">
+        <v>247.98</v>
+      </c>
+      <c r="D8" s="48" t="n">
+        <v>297.58</v>
+      </c>
+      <c r="E8" s="50" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>22.0x × FY26E EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Analyst consensus 12mo target</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="n">
+        <v>275</v>
+      </c>
+      <c r="C9" s="48" t="n">
+        <v>379.55</v>
+      </c>
+      <c r="D9" s="48" t="n">
+        <v>425</v>
+      </c>
+      <c r="E9" s="50" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>22 analysts | Buys: 22 / Sells: 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>Weighted blended target</t>
+        </is>
+      </c>
+      <c r="B11" s="51" t="n">
+        <v>259.28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>FINAL PRICE TARGET &amp; RECOMMENDATION</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>12-month price target</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Current stock price</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>338.19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>Implied upside</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="n">
+        <v>0.1827670835920636</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="36" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="B17" s="52" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B18" s="53" t="inlineStr">
+        <is>
+          <t>12mo PT $400 ($395-$405). 18% upside. Anchored to ~45x FY27E non-GAAP EPS of $9.10.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5448,4 +6415,1045 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Cadence (CDNS) – DCF Valuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Valuation date: 2026-05-20 | Stock: $338.19 | Market cap: $93.3B | EV: $92.7B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>UNLEVERED FCF BUILD ($M)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>6175</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>7035</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>7950</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>8830</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>9685</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>10024</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>EBIT (operating income)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>2748</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>3187</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>3657</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>4106</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>4552</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>4711</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>NOPAT (× (1-21%))</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="n">
+        <v>2171</v>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>2518</v>
+      </c>
+      <c r="D8" s="32" t="n">
+        <v>2889</v>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>3244</v>
+      </c>
+      <c r="F8" s="32" t="n">
+        <v>3596</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>+ D&amp;A</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>309</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>352</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>398</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>442</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>484</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>- Capex</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>-167</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>-190</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>-215</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-238</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>-261</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>-270</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>- Δ Working capital</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>-93</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>-106</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>-119</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-132</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>-145</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>-150</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Unlevered FCF</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="n">
+        <v>2220</v>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>2574</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>2953</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>3314</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <v>3674</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>3803</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PRESENT VALUE OF FCF</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Discount factor (WACC=9.4%)</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="n">
+        <v>0.9143262581243603</v>
+      </c>
+      <c r="C15" s="33" t="n">
+        <v>0.8359925062956944</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>0.7643699001013481</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>0.6988834705825567</v>
+      </c>
+      <c r="F15" s="33" t="n">
+        <v>0.6390075085227156</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>PV of UFCF</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n">
+        <v>2030</v>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>2152</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>2257</v>
+      </c>
+      <c r="E16" s="32" t="n">
+        <v>2316</v>
+      </c>
+      <c r="F16" s="32" t="n">
+        <v>2348</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>Sum PV of explicit FCFs</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="n">
+        <v>11103</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>TERMINAL VALUE</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Terminal FCF (FY30 × (1+g))</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>3803</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>Terminal growth (g)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>0.09370149999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Terminal value (Gordon)</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>64778</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>41394</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>ENTERPRISE &amp; EQUITY VALUE</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>Enterprise value ($M)</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="n">
+        <v>52497</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>(+) Cash &amp; short-term investments</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>(-) Total debt</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>-2480</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>Equity value ($M)</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="n">
+        <v>53017</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>Diluted shares (M)</t>
+        </is>
+      </c>
+      <c r="B31" s="37" t="n">
+        <v>273.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>DCF value per share</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="n">
+        <v>193.99</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>Current stock price</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>338.19</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="36" t="inlineStr">
+        <is>
+          <t>Implied upside / (downside)</t>
+        </is>
+      </c>
+      <c r="B34" s="39" t="n">
+        <v>-0.4263975749557308</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>WACC BUILD</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Risk-free rate (10y UST)</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Equity risk premium</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>Beta (5y monthly)</t>
+        </is>
+      </c>
+      <c r="B39" s="37" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>Cost of equity (CAPM)</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>0.0955</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>Pre-tax cost of debt</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>After-tax cost of debt</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>0.03555</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>Debt / Capital</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>Equity / Capital</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="36" t="inlineStr">
+        <is>
+          <t>WACC</t>
+        </is>
+      </c>
+      <c r="B45" s="39" t="n">
+        <v>0.09370149999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Cadence (CDNS) – DCF Sensitivity Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DCF value per share — sensitivity to WACC and terminal growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="40" t="inlineStr">
+        <is>
+          <t>Terminal growth ↓ / WACC →</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>8.4%</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>2.0%</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="n">
+        <v>204.23</v>
+      </c>
+      <c r="C5" s="42" t="n">
+        <v>187.71</v>
+      </c>
+      <c r="D5" s="42" t="n">
+        <v>173.6</v>
+      </c>
+      <c r="E5" s="42" t="n">
+        <v>161.41</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>150.78</v>
+      </c>
+      <c r="G5" s="42" t="n">
+        <v>141.44</v>
+      </c>
+      <c r="H5" s="42" t="n">
+        <v>133.15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="n">
+        <v>219.98</v>
+      </c>
+      <c r="C6" s="42" t="n">
+        <v>200.74</v>
+      </c>
+      <c r="D6" s="42" t="n">
+        <v>184.53</v>
+      </c>
+      <c r="E6" s="42" t="n">
+        <v>170.69</v>
+      </c>
+      <c r="F6" s="42" t="n">
+        <v>158.74</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <v>148.31</v>
+      </c>
+      <c r="H6" s="42" t="n">
+        <v>139.14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>3.0%</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="n">
+        <v>238.96</v>
+      </c>
+      <c r="C7" s="42" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="D7" s="42" t="n">
+        <v>197.32</v>
+      </c>
+      <c r="E7" s="42" t="n">
+        <v>181.42</v>
+      </c>
+      <c r="F7" s="42" t="n">
+        <v>167.85</v>
+      </c>
+      <c r="G7" s="42" t="n">
+        <v>156.12</v>
+      </c>
+      <c r="H7" s="42" t="n">
+        <v>145.89</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>3.5%</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="n">
+        <v>262.29</v>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>234.83</v>
+      </c>
+      <c r="D8" s="42" t="n">
+        <v>212.5</v>
+      </c>
+      <c r="E8" s="42" t="n">
+        <v>193.99</v>
+      </c>
+      <c r="F8" s="42" t="n">
+        <v>178.39</v>
+      </c>
+      <c r="G8" s="42" t="n">
+        <v>165.07</v>
+      </c>
+      <c r="H8" s="42" t="n">
+        <v>153.56</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="n">
+        <v>291.64</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <v>257.73</v>
+      </c>
+      <c r="D9" s="42" t="n">
+        <v>230.8</v>
+      </c>
+      <c r="E9" s="42" t="n">
+        <v>208.89</v>
+      </c>
+      <c r="F9" s="42" t="n">
+        <v>190.72</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <v>175.42</v>
+      </c>
+      <c r="H9" s="42" t="n">
+        <v>162.35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>IMPLIED UPSIDE / DOWNSIDE vs. current stock</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Terminal growth ↓ / WACC →</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>8.4%</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="H13" s="41" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>2.0%</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>-0.3961063192953953</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>-0.4449682365223776</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>-0.4866865993744616</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>-0.5227159752175883</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>-0.5541412714891045</v>
+      </c>
+      <c r="G14" s="30" t="n">
+        <v>-0.5817881464613113</v>
+      </c>
+      <c r="H14" s="30" t="n">
+        <v>-0.6062960776291851</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>-0.3495404176280155</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>-0.4064318306797399</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>-0.4543601802483993</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>-0.4952831216264663</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>-0.5306270526093573</v>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>-0.5614558711836199</v>
+      </c>
+      <c r="H15" s="30" t="n">
+        <v>-0.5885792476516507</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>3.0%</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>-0.293413023672435</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <v>-0.3607193858358381</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>-0.4165268457750181</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>-0.4635437990210945</v>
+      </c>
+      <c r="F16" s="30" t="n">
+        <v>-0.503690169176471</v>
+      </c>
+      <c r="G16" s="30" t="n">
+        <v>-0.5383648630066402</v>
+      </c>
+      <c r="H16" s="30" t="n">
+        <v>-0.5686112750685071</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>3.5%</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
+        <v>-0.2244422733204884</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <v>-0.3056206911138214</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>-0.3716483944104179</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>-0.4263975749557308</v>
+      </c>
+      <c r="F17" s="30" t="n">
+        <v>-0.4725246752033486</v>
+      </c>
+      <c r="G17" s="30" t="n">
+        <v>-0.5119127916538957</v>
+      </c>
+      <c r="H17" s="30" t="n">
+        <v>-0.5459339990677743</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>4.0%</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>-0.1376503143973115</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>-0.2379140321978942</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>-0.3175549391209691</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>-0.3823341839461731</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>-0.436050033427679</v>
+      </c>
+      <c r="G18" s="30" t="n">
+        <v>-0.4813082166155638</v>
+      </c>
+      <c r="H18" s="30" t="n">
+        <v>-0.5199558816005916</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5:H9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14:H18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>